<commit_message>
Fix timezone-dependent plan start date parsing
</commit_message>
<xml_diff>
--- a/fixtures/money-plan.xlsx
+++ b/fixtures/money-plan.xlsx
@@ -64,9 +64,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -441,8 +440,8 @@
       <c r="A7" t="str">
         <v>Plan start month</v>
       </c>
-      <c r="B7" s="1" t="d">
-        <v>2026-09-30T16:00:00.000Z</v>
+      <c r="B7">
+        <v>46296</v>
       </c>
     </row>
     <row r="8">

</xml_diff>